<commit_message>
Objects named the way the dissertation names them, and the site rebuilt
lamppost -> lamp post, bus-stop sign -> bus stop sign in the results
table; the site builders follow. Also the duplicated line in the LoD95
note, and deploy_site.sh, which publishes site/ to gh-pages through a
throwaway worktree. The dissertation drafts in docs/thesis/ are ignored.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tables/capture_comparison_summary.xlsx
+++ b/docs/tables/capture_comparison_summary.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X13"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -469,11 +469,12 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -574,25 +575,30 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>images in</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>reg-rate (%)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>points raw</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>points density-matched</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>excluded as gap</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>DBSCAN (ft/eps/mp)</t>
         </is>
@@ -665,18 +671,21 @@
         <v>1.3</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V2" s="2" t="n">
         <v>105933</v>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="W2" s="2" t="n">
         <v>3847</v>
       </c>
-      <c r="W2" s="2" t="n">
+      <c r="X2" s="2" t="n">
         <v>754</v>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -749,18 +758,21 @@
         <v>1.11</v>
       </c>
       <c r="T3" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U3" t="n">
+        <v>100</v>
+      </c>
+      <c r="V3" t="n">
         <v>36609</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>2715</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>419</v>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -833,18 +845,21 @@
         <v>1.42</v>
       </c>
       <c r="T4" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U4" t="n">
+        <v>100</v>
+      </c>
+      <c r="V4" t="n">
         <v>167287</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>5592</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>1295</v>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -917,18 +932,21 @@
         <v>1.27</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V5" s="2" t="n">
         <v>441241</v>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="W5" s="2" t="n">
         <v>16196</v>
       </c>
-      <c r="W5" s="2" t="n">
+      <c r="X5" s="2" t="n">
         <v>4072</v>
       </c>
-      <c r="X5" s="2" t="inlineStr">
+      <c r="Y5" s="2" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1001,18 +1019,21 @@
         <v>1.21</v>
       </c>
       <c r="T6" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U6" t="n">
+        <v>100</v>
+      </c>
+      <c r="V6" t="n">
         <v>750396</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>12872</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>2676</v>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1085,18 +1106,21 @@
         <v>1.38</v>
       </c>
       <c r="T7" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="U7" t="n">
+        <v>100</v>
+      </c>
+      <c r="V7" t="n">
         <v>482225</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>13029</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>2580</v>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1169,18 +1193,21 @@
         <v>1.74</v>
       </c>
       <c r="T8" s="2" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="U8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V8" s="2" t="n">
         <v>547654</v>
       </c>
-      <c r="V8" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>25404</v>
       </c>
-      <c r="W8" s="2" t="n">
+      <c r="X8" s="2" t="n">
         <v>14198</v>
       </c>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="Y8" s="2" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1253,18 +1280,21 @@
         <v>1.95</v>
       </c>
       <c r="T9" t="n">
+        <v>48</v>
+      </c>
+      <c r="U9" t="n">
         <v>95.8</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>801528</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>19421</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>15582</v>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1337,18 +1367,21 @@
         <v>1.96</v>
       </c>
       <c r="T10" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="U10" t="n">
+        <v>100</v>
+      </c>
+      <c r="V10" t="n">
         <v>716317</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>35676</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>21922</v>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1421,18 +1454,21 @@
         <v>1.73</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="U11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="V11" s="2" t="n">
         <v>540530</v>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="W11" s="2" t="n">
         <v>75146</v>
       </c>
-      <c r="W11" s="2" t="n">
+      <c r="X11" s="2" t="n">
         <v>36753</v>
       </c>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="Y11" s="2" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1505,18 +1541,21 @@
         <v>1.91</v>
       </c>
       <c r="T12" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="U12" t="n">
+        <v>100</v>
+      </c>
+      <c r="V12" t="n">
         <v>1129311</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>70386</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>49235</v>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -1589,18 +1628,21 @@
         <v>1.65</v>
       </c>
       <c r="T13" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="U13" t="n">
+        <v>100</v>
+      </c>
+      <c r="V13" t="n">
         <v>484330</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>59039</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>28083</v>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>

</xml_diff>